<commit_message>
updated pipeline standardization of names
</commit_message>
<xml_diff>
--- a/data/processed/website_clean.xlsx
+++ b/data/processed/website_clean.xlsx
@@ -3110,12 +3110,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Art jason Luzande</t>
+          <t>Art Jason Luzande</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Art jason Luzande</t>
+          <t>Art Jason Luzande</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3161,7 +3161,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Art jason Luzande</t>
+          <t>Art Jason Luzande</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3830,12 +3830,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -4724,12 +4724,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4775,7 +4775,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5076,12 +5076,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -5523,12 +5523,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P57" t="inlineStr">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -6270,7 +6270,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="P65" t="inlineStr">
@@ -7536,12 +7536,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="P84" t="inlineStr">
@@ -8153,12 +8153,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>CHRISTOPER TATEL</t>
+          <t>Christoper Tatel</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>CHRISTOPER TATEL</t>
+          <t>Christoper Tatel</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -8204,7 +8204,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>CHRISTOPER TATEL</t>
+          <t>Christoper Tatel</t>
         </is>
       </c>
       <c r="P91" t="inlineStr">
@@ -9569,12 +9569,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -9620,7 +9620,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="P107" t="inlineStr">
@@ -9921,12 +9921,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="P111" t="inlineStr">
@@ -10368,12 +10368,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -10419,7 +10419,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -11064,12 +11064,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -11115,7 +11115,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>johan miguel guasch</t>
+          <t>Johan Miguel Guasch</t>
         </is>
       </c>
       <c r="P124" t="inlineStr">
@@ -12571,12 +12571,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>samantha nogales</t>
+          <t>Samantha Nogales</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>samantha nogales</t>
+          <t>Samantha Nogales</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -12622,7 +12622,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>samantha nogales</t>
+          <t>Samantha Nogales</t>
         </is>
       </c>
       <c r="P141" t="inlineStr">
@@ -14576,12 +14576,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -14627,7 +14627,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P164" t="inlineStr">
@@ -15193,12 +15193,12 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -15244,7 +15244,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
@@ -17471,12 +17471,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>GILBERT DOMINGO VIDANES</t>
+          <t>Gilbert Domingo Vidanes</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>GILBERT DOMINGO VIDANES</t>
+          <t>Gilbert Domingo Vidanes</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -17522,7 +17522,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>GILBERT DOMINGO VIDANES</t>
+          <t>Gilbert Domingo Vidanes</t>
         </is>
       </c>
       <c r="P197" t="inlineStr">
@@ -20299,12 +20299,12 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>OLIVE LANCIN</t>
+          <t>Olive Lancin</t>
         </is>
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>OLIVE LANCIN</t>
+          <t>Olive Lancin</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -20350,7 +20350,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>HARVEY VALENCIA</t>
+          <t>Harvey Valencia</t>
         </is>
       </c>
       <c r="P229" t="inlineStr">
@@ -20386,12 +20386,12 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>OLIVE LANCIN</t>
+          <t>Olive Lancin</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>OLIVE LANCIN</t>
+          <t>Olive Lancin</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -20437,7 +20437,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>HARVEY VALENCIA</t>
+          <t>Harvey Valencia</t>
         </is>
       </c>
       <c r="P230" t="inlineStr">
@@ -21782,12 +21782,12 @@
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>NOL SHEANLI HARANI</t>
+          <t>Nol Sheanli Harani</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>NOL SHEANLI HARANI</t>
+          <t>Nol Sheanli Harani</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -21833,7 +21833,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>NOL SHEANLI HARANI</t>
+          <t>Nol Sheanli Harani</t>
         </is>
       </c>
       <c r="P246" t="inlineStr">
@@ -21960,12 +21960,12 @@
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -22011,7 +22011,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P248" t="inlineStr">
@@ -23004,12 +23004,12 @@
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -23055,7 +23055,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
@@ -23526,12 +23526,12 @@
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>samantha nogales</t>
+          <t>Samantha Nogales</t>
         </is>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>samantha nogales</t>
+          <t>Samantha Nogales</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -23577,7 +23577,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>samantha nogales</t>
+          <t>Samantha Nogales</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
@@ -24222,12 +24222,12 @@
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>EDWIN IAN MELCHOR</t>
+          <t>Edwin Ian Melchor</t>
         </is>
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>EDWIN IAN MELCHOR</t>
+          <t>Edwin Ian Melchor</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -24273,7 +24273,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>EDWIN IAN MELCHOR</t>
+          <t>Edwin Ian Melchor</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
@@ -24396,12 +24396,12 @@
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>MARC MANLIGUEZ</t>
+          <t>Marc Manliguez</t>
         </is>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>MARC MANLIGUEZ</t>
+          <t>Marc Manliguez</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -24447,7 +24447,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>MARC MANLIGUEZ</t>
+          <t>Marc Manliguez</t>
         </is>
       </c>
       <c r="P276" t="inlineStr">
@@ -24744,12 +24744,12 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -24795,7 +24795,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="P280" t="inlineStr">
@@ -24922,12 +24922,12 @@
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>EL CID PAOLO RUIZ</t>
+          <t>El Cid Paolo Ruiz</t>
         </is>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>EL CID PAOLO RUIZ</t>
+          <t>El Cid Paolo Ruiz</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -24973,7 +24973,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>EL CID PAOLO RUIZ</t>
+          <t>El Cid Paolo Ruiz</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
@@ -25100,12 +25100,12 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>ARJON BRIX TEBERIO</t>
+          <t>Arjon Brix Teberio</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>ARJON BRIX TEBERIO</t>
+          <t>Arjon Brix Teberio</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -25151,7 +25151,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>ARJON BRIX TEBERIO</t>
+          <t>Arjon Brix Teberio</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -27026,12 +27026,12 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -27077,7 +27077,7 @@
       </c>
       <c r="O306" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P306" t="inlineStr">
@@ -27726,12 +27726,12 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>khearl Mark Corvera</t>
+          <t>Khearl Mark Corvera</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>khearl Mark Corvera</t>
+          <t>Khearl Mark Corvera</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -27777,7 +27777,7 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>khearl Mark Corvera</t>
+          <t>Khearl Mark Corvera</t>
         </is>
       </c>
       <c r="P314" t="inlineStr">
@@ -30712,12 +30712,12 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -30763,7 +30763,7 @@
       </c>
       <c r="O348" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P348" t="inlineStr">
@@ -30799,12 +30799,12 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>mary jane diaz</t>
+          <t>Mary Jane Diaz</t>
         </is>
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>mary jane diaz</t>
+          <t>Mary Jane Diaz</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
@@ -30850,7 +30850,7 @@
       </c>
       <c r="O349" t="inlineStr">
         <is>
-          <t>mary jane diaz</t>
+          <t>Mary Jane Diaz</t>
         </is>
       </c>
       <c r="P349" t="inlineStr">
@@ -32982,12 +32982,12 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
@@ -33033,7 +33033,7 @@
       </c>
       <c r="O374" t="inlineStr">
         <is>
-          <t>Eric Ta-aca</t>
+          <t>Eric Ta-Aca</t>
         </is>
       </c>
       <c r="P374" t="inlineStr">
@@ -33243,12 +33243,12 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Leslee nadyne Cruz</t>
+          <t>Leslee Nadyne Cruz</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Leslee nadyne Cruz</t>
+          <t>Leslee Nadyne Cruz</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -36241,12 +36241,12 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
@@ -36292,7 +36292,7 @@
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t>RV Henretty-Jornales</t>
+          <t>Rv Henretty-Jornales</t>
         </is>
       </c>
       <c r="P411" t="inlineStr">
@@ -37028,12 +37028,12 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>iann Villanueva</t>
+          <t>Iann Villanueva</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>iann Villanueva</t>
+          <t>Iann Villanueva</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
@@ -38689,12 +38689,12 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
@@ -38740,7 +38740,7 @@
       </c>
       <c r="O439" t="inlineStr">
         <is>
-          <t>RYAN NEIL SELOTERIO</t>
+          <t>Ryan Neil Seloterio</t>
         </is>
       </c>
       <c r="P439" t="inlineStr">
@@ -39733,12 +39733,12 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F451" t="inlineStr">
@@ -39784,7 +39784,7 @@
       </c>
       <c r="O451" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P451" t="inlineStr">
@@ -39998,12 +39998,12 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Art jason Luzande</t>
+          <t>Art Jason Luzande</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>Art jason Luzande</t>
+          <t>Art Jason Luzande</t>
         </is>
       </c>
       <c r="F454" t="inlineStr">
@@ -40049,7 +40049,7 @@
       </c>
       <c r="O454" t="inlineStr">
         <is>
-          <t>Art jason Luzande</t>
+          <t>Art Jason Luzande</t>
         </is>
       </c>
       <c r="P454" t="inlineStr">
@@ -41216,12 +41216,12 @@
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="F468" t="inlineStr">
@@ -41267,7 +41267,7 @@
       </c>
       <c r="O468" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="P468" t="inlineStr">
@@ -41303,12 +41303,12 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="F469" t="inlineStr">
@@ -41354,7 +41354,7 @@
       </c>
       <c r="O469" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="P469" t="inlineStr">
@@ -41390,12 +41390,12 @@
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="F470" t="inlineStr">
@@ -41441,7 +41441,7 @@
       </c>
       <c r="O470" t="inlineStr">
         <is>
-          <t>ERVIN JOHN SERNA</t>
+          <t>Ervin John Serna</t>
         </is>
       </c>
       <c r="P470" t="inlineStr">
@@ -42612,12 +42612,12 @@
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>ARLAN FERNANDEZ</t>
+          <t>Arlan Fernandez</t>
         </is>
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>ARLAN FERNANDEZ</t>
+          <t>Arlan Fernandez</t>
         </is>
       </c>
       <c r="F484" t="inlineStr">
@@ -42663,7 +42663,7 @@
       </c>
       <c r="O484" t="inlineStr">
         <is>
-          <t>ARLAN FERNANDEZ</t>
+          <t>Arlan Fernandez</t>
         </is>
       </c>
       <c r="P484" t="inlineStr">
@@ -43838,12 +43838,12 @@
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>iann Villanueva</t>
+          <t>Iann Villanueva</t>
         </is>
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>iann Villanueva</t>
+          <t>Iann Villanueva</t>
         </is>
       </c>
       <c r="F498" t="inlineStr">
@@ -45147,12 +45147,12 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>Leslee nadyne Cruz</t>
+          <t>Leslee Nadyne Cruz</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>Leslee nadyne Cruz</t>
+          <t>Leslee Nadyne Cruz</t>
         </is>
       </c>
       <c r="F513" t="inlineStr">
@@ -46646,12 +46646,12 @@
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>mary jane diaz</t>
+          <t>Mary Jane Diaz</t>
         </is>
       </c>
       <c r="E530" t="inlineStr">
         <is>
-          <t>mary jane diaz</t>
+          <t>Mary Jane Diaz</t>
         </is>
       </c>
       <c r="F530" t="inlineStr">
@@ -46697,7 +46697,7 @@
       </c>
       <c r="O530" t="inlineStr">
         <is>
-          <t>mary jane diaz</t>
+          <t>Mary Jane Diaz</t>
         </is>
       </c>
       <c r="P530" t="inlineStr">
@@ -49276,12 +49276,12 @@
       </c>
       <c r="D560" t="inlineStr">
         <is>
-          <t>JOHN CHRISTIAN Sagun</t>
+          <t>John Christian Sagun</t>
         </is>
       </c>
       <c r="E560" t="inlineStr">
         <is>
-          <t>JOHN CHRISTIAN Sagun</t>
+          <t>John Christian Sagun</t>
         </is>
       </c>
       <c r="F560" t="inlineStr">
@@ -49327,7 +49327,7 @@
       </c>
       <c r="O560" t="inlineStr">
         <is>
-          <t>JOHN CHRISTIAN Sagun</t>
+          <t>John Christian Sagun</t>
         </is>
       </c>
       <c r="P560" t="inlineStr">
@@ -50063,12 +50063,12 @@
       </c>
       <c r="D569" t="inlineStr">
         <is>
-          <t>JOEL INARSOLIN</t>
+          <t>Joel Inarsolin</t>
         </is>
       </c>
       <c r="E569" t="inlineStr">
         <is>
-          <t>JOEL INARSOLIN</t>
+          <t>Joel Inarsolin</t>
         </is>
       </c>
       <c r="F569" t="inlineStr">
@@ -50114,7 +50114,7 @@
       </c>
       <c r="O569" t="inlineStr">
         <is>
-          <t>JOEL INARSOLIN</t>
+          <t>Joel Inarsolin</t>
         </is>
       </c>
       <c r="P569" t="inlineStr">
@@ -52503,12 +52503,12 @@
       </c>
       <c r="D597" t="inlineStr">
         <is>
-          <t>Dan Roniel CASIA</t>
+          <t>Dan Roniel Casia</t>
         </is>
       </c>
       <c r="E597" t="inlineStr">
         <is>
-          <t>Dan Roniel CASIA</t>
+          <t>Dan Roniel Casia</t>
         </is>
       </c>
       <c r="F597" t="inlineStr">
@@ -52554,7 +52554,7 @@
       </c>
       <c r="O597" t="inlineStr">
         <is>
-          <t>Dan Roniel CASIA</t>
+          <t>Dan Roniel Casia</t>
         </is>
       </c>
       <c r="P597" t="inlineStr">
@@ -53729,12 +53729,12 @@
       </c>
       <c r="D611" t="inlineStr">
         <is>
-          <t>MASATOSHI OGASAWARA</t>
+          <t>Masatoshi Ogasawara</t>
         </is>
       </c>
       <c r="E611" t="inlineStr">
         <is>
-          <t>MASATOSHI OGASAWARA</t>
+          <t>Masatoshi Ogasawara</t>
         </is>
       </c>
       <c r="F611" t="inlineStr">
@@ -53780,7 +53780,7 @@
       </c>
       <c r="O611" t="inlineStr">
         <is>
-          <t>MASATOSHI OGASAWARA</t>
+          <t>Masatoshi Ogasawara</t>
         </is>
       </c>
       <c r="P611" t="inlineStr">
@@ -54516,12 +54516,12 @@
       </c>
       <c r="D620" t="inlineStr">
         <is>
-          <t>EL CID PAOLO RUIZ</t>
+          <t>El Cid Paolo Ruiz</t>
         </is>
       </c>
       <c r="E620" t="inlineStr">
         <is>
-          <t>EL CID PAOLO RUIZ</t>
+          <t>El Cid Paolo Ruiz</t>
         </is>
       </c>
       <c r="F620" t="inlineStr">
@@ -54567,7 +54567,7 @@
       </c>
       <c r="O620" t="inlineStr">
         <is>
-          <t>EL CID PAOLO RUIZ</t>
+          <t>El Cid Paolo Ruiz</t>
         </is>
       </c>
       <c r="P620" t="inlineStr">
@@ -55394,12 +55394,12 @@
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E630" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F630" t="inlineStr">
@@ -55445,7 +55445,7 @@
       </c>
       <c r="O630" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P630" t="inlineStr">
@@ -56351,12 +56351,12 @@
       </c>
       <c r="D641" t="inlineStr">
         <is>
-          <t>ANGELICA VICUNA</t>
+          <t>Angelica Vicuna</t>
         </is>
       </c>
       <c r="E641" t="inlineStr">
         <is>
-          <t>ANGELICA VICUNA</t>
+          <t>Angelica Vicuna</t>
         </is>
       </c>
       <c r="F641" t="inlineStr">
@@ -56402,7 +56402,7 @@
       </c>
       <c r="O641" t="inlineStr">
         <is>
-          <t>ANGELICA VICUNA</t>
+          <t>Angelica Vicuna</t>
         </is>
       </c>
       <c r="P641" t="inlineStr">
@@ -56438,12 +56438,12 @@
       </c>
       <c r="D642" t="inlineStr">
         <is>
-          <t>GILBERT DOMINGO VIDANES</t>
+          <t>Gilbert Domingo Vidanes</t>
         </is>
       </c>
       <c r="E642" t="inlineStr">
         <is>
-          <t>GILBERT DOMINGO VIDANES</t>
+          <t>Gilbert Domingo Vidanes</t>
         </is>
       </c>
       <c r="F642" t="inlineStr">
@@ -56489,7 +56489,7 @@
       </c>
       <c r="O642" t="inlineStr">
         <is>
-          <t>GILBERT DOMINGO VIDANES</t>
+          <t>Gilbert Domingo Vidanes</t>
         </is>
       </c>
       <c r="P642" t="inlineStr">
@@ -56525,12 +56525,12 @@
       </c>
       <c r="D643" t="inlineStr">
         <is>
-          <t>KIMBERLY FAITH YTAC</t>
+          <t>Kimberly Faith Ytac</t>
         </is>
       </c>
       <c r="E643" t="inlineStr">
         <is>
-          <t>KIMBERLY FAITH YTAC</t>
+          <t>Kimberly Faith Ytac</t>
         </is>
       </c>
       <c r="F643" t="inlineStr">
@@ -56576,7 +56576,7 @@
       </c>
       <c r="O643" t="inlineStr">
         <is>
-          <t>KIMBERLY FAITH YTAC</t>
+          <t>Kimberly Faith Ytac</t>
         </is>
       </c>
       <c r="P643" t="inlineStr">
@@ -56616,12 +56616,12 @@
       </c>
       <c r="D644" t="inlineStr">
         <is>
-          <t>mark tan</t>
+          <t>Mark Tan</t>
         </is>
       </c>
       <c r="E644" t="inlineStr">
         <is>
-          <t>mark tan</t>
+          <t>Mark Tan</t>
         </is>
       </c>
       <c r="F644" t="inlineStr">
@@ -56667,7 +56667,7 @@
       </c>
       <c r="O644" t="inlineStr">
         <is>
-          <t>mark tan</t>
+          <t>Mark Tan</t>
         </is>
       </c>
       <c r="P644" t="inlineStr">
@@ -58720,12 +58720,12 @@
       </c>
       <c r="D668" t="inlineStr">
         <is>
-          <t>ARLAN FERNANDEZ</t>
+          <t>Arlan Fernandez</t>
         </is>
       </c>
       <c r="E668" t="inlineStr">
         <is>
-          <t>ARLAN FERNANDEZ</t>
+          <t>Arlan Fernandez</t>
         </is>
       </c>
       <c r="F668" t="inlineStr">
@@ -58771,7 +58771,7 @@
       </c>
       <c r="O668" t="inlineStr">
         <is>
-          <t>ARLAN FERNANDEZ</t>
+          <t>Arlan Fernandez</t>
         </is>
       </c>
       <c r="P668" t="inlineStr">
@@ -63794,12 +63794,12 @@
       </c>
       <c r="D726" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="E726" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="F726" t="inlineStr">
@@ -63845,7 +63845,7 @@
       </c>
       <c r="O726" t="inlineStr">
         <is>
-          <t>FRANCIS RYAN UY</t>
+          <t>Francis Ryan Uy</t>
         </is>
       </c>
       <c r="P726" t="inlineStr">
@@ -66246,12 +66246,12 @@
       </c>
       <c r="D754" t="inlineStr">
         <is>
-          <t>Mohammed ABDULLAH</t>
+          <t>Mohammed Abdullah</t>
         </is>
       </c>
       <c r="E754" t="inlineStr">
         <is>
-          <t>Mohammed ABDULLAH</t>
+          <t>Mohammed Abdullah</t>
         </is>
       </c>
       <c r="F754" t="inlineStr">
@@ -66297,7 +66297,7 @@
       </c>
       <c r="O754" t="inlineStr">
         <is>
-          <t>Mohammed ABDULLAH</t>
+          <t>Mohammed Abdullah</t>
         </is>
       </c>
       <c r="P754" t="inlineStr">
@@ -66511,12 +66511,12 @@
       </c>
       <c r="D757" t="inlineStr">
         <is>
-          <t>HANNAH LINCHANGCO</t>
+          <t>Hannah Linchangco</t>
         </is>
       </c>
       <c r="E757" t="inlineStr">
         <is>
-          <t>HANNAH LINCHANGCO</t>
+          <t>Hannah Linchangco</t>
         </is>
       </c>
       <c r="F757" t="inlineStr">
@@ -66562,7 +66562,7 @@
       </c>
       <c r="O757" t="inlineStr">
         <is>
-          <t>HANNAH LINCHANGCO</t>
+          <t>Hannah Linchangco</t>
         </is>
       </c>
       <c r="P757" t="inlineStr">
@@ -67646,12 +67646,12 @@
       </c>
       <c r="D770" t="inlineStr">
         <is>
-          <t>JAN KYLE BALORAN</t>
+          <t>Jan Kyle Baloran</t>
         </is>
       </c>
       <c r="E770" t="inlineStr">
         <is>
-          <t>JAN KYLE BALORAN</t>
+          <t>Jan Kyle Baloran</t>
         </is>
       </c>
       <c r="F770" t="inlineStr">
@@ -67697,7 +67697,7 @@
       </c>
       <c r="O770" t="inlineStr">
         <is>
-          <t>JAN KYLE BALORAN</t>
+          <t>Jan Kyle Baloran</t>
         </is>
       </c>
       <c r="P770" t="inlineStr">
@@ -67820,12 +67820,12 @@
       </c>
       <c r="D772" t="inlineStr">
         <is>
-          <t>Roumell SO</t>
+          <t>Roumell So</t>
         </is>
       </c>
       <c r="E772" t="inlineStr">
         <is>
-          <t>Roumell SO</t>
+          <t>Roumell So</t>
         </is>
       </c>
       <c r="F772" t="inlineStr">
@@ -67871,7 +67871,7 @@
       </c>
       <c r="O772" t="inlineStr">
         <is>
-          <t>Roumell SO</t>
+          <t>Roumell So</t>
         </is>
       </c>
       <c r="P772" t="inlineStr">
@@ -68346,12 +68346,12 @@
       </c>
       <c r="D778" t="inlineStr">
         <is>
-          <t>Christopher SANTOS</t>
+          <t>Christopher Santos</t>
         </is>
       </c>
       <c r="E778" t="inlineStr">
         <is>
-          <t>Christopher SANTOS</t>
+          <t>Christopher Santos</t>
         </is>
       </c>
       <c r="F778" t="inlineStr">
@@ -68397,7 +68397,7 @@
       </c>
       <c r="O778" t="inlineStr">
         <is>
-          <t>Christopher SANTOS</t>
+          <t>Christopher Santos</t>
         </is>
       </c>
       <c r="P778" t="inlineStr">
@@ -69920,12 +69920,12 @@
       </c>
       <c r="D796" t="inlineStr">
         <is>
-          <t>angel jen belicena</t>
+          <t>Angel Jen Belicena</t>
         </is>
       </c>
       <c r="E796" t="inlineStr">
         <is>
-          <t>angel jen belicena</t>
+          <t>Angel Jen Belicena</t>
         </is>
       </c>
       <c r="F796" t="inlineStr">
@@ -69971,7 +69971,7 @@
       </c>
       <c r="O796" t="inlineStr">
         <is>
-          <t>angel jen belicena</t>
+          <t>Angel Jen Belicena</t>
         </is>
       </c>
       <c r="P796" t="inlineStr">

</xml_diff>